<commit_message>
Improvised CV code with excel sheets and trace files
</commit_message>
<xml_diff>
--- a/pages/STPTestData.xlsx
+++ b/pages/STPTestData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Serole Automation\playwright_python\pages\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D84D6713-D809-4B9A-83B1-68BA90C84B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95EA2593-B9B0-4D17-9F77-6B49D3BF36FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{45C1E7C0-1AF2-45CB-BEA8-DD612E61CE1D}"/>
   </bookViews>
@@ -804,10 +804,10 @@
       <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>34</v>
       </c>
       <c r="C17" s="1" t="s">

</xml_diff>

<commit_message>
18/03: CV and PA quote completed successfully
</commit_message>
<xml_diff>
--- a/pages/STPTestData.xlsx
+++ b/pages/STPTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95EA2593-B9B0-4D17-9F77-6B49D3BF36FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BFD6B6-EA1A-4765-93D1-3DD56A829C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{45C1E7C0-1AF2-45CB-BEA8-DD612E61CE1D}"/>
   </bookViews>
@@ -816,10 +816,10 @@
       <c r="D17" s="1"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C18" s="1" t="s">
@@ -828,10 +828,10 @@
       <c r="D18" s="1"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>38</v>
       </c>
       <c r="C19" s="1" t="s">

</xml_diff>

<commit_message>
PA changes and MC added
</commit_message>
<xml_diff>
--- a/pages/STPTestData.xlsx
+++ b/pages/STPTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BFD6B6-EA1A-4765-93D1-3DD56A829C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0CEE9E6-CF00-4D9D-BECC-5EDE102763C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{45C1E7C0-1AF2-45CB-BEA8-DD612E61CE1D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="79">
   <si>
     <t>RegNo</t>
   </si>
@@ -48,9 +48,6 @@
     <t>740504-12-5338</t>
   </si>
   <si>
-    <t>Coverage Type</t>
-  </si>
-  <si>
     <t>PDH3345</t>
   </si>
   <si>
@@ -160,13 +157,127 @@
   </si>
   <si>
     <t xml:space="preserve">CV C </t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>MC</t>
+  </si>
+  <si>
+    <t>AHX2629</t>
+  </si>
+  <si>
+    <t>WTG8948</t>
+  </si>
+  <si>
+    <t>VKJ8276</t>
+  </si>
+  <si>
+    <t>970421-01-6682</t>
+  </si>
+  <si>
+    <t>WNB1173</t>
+  </si>
+  <si>
+    <t>841118-03-5599</t>
+  </si>
+  <si>
+    <t>750103-03-6915</t>
+  </si>
+  <si>
+    <t>730614-08-6537</t>
+  </si>
+  <si>
+    <t>AGT658</t>
+  </si>
+  <si>
+    <t>681008-08-6061</t>
+  </si>
+  <si>
+    <t>KCW4068</t>
+  </si>
+  <si>
+    <t>680731-02-5263</t>
+  </si>
+  <si>
+    <t>MDA5074</t>
+  </si>
+  <si>
+    <t>841229-04-5386</t>
+  </si>
+  <si>
+    <t>PNE1087</t>
+  </si>
+  <si>
+    <t>800929-07-5681</t>
+  </si>
+  <si>
+    <t>TCW4312</t>
+  </si>
+  <si>
+    <t>060410-11-0259</t>
+  </si>
+  <si>
+    <t>VMF1335</t>
+  </si>
+  <si>
+    <t>790620-08-6060</t>
+  </si>
+  <si>
+    <t>BQS5741</t>
+  </si>
+  <si>
+    <t>980720-03-6412</t>
+  </si>
+  <si>
+    <t>VKM4162</t>
+  </si>
+  <si>
+    <t>030105-10-0559</t>
+  </si>
+  <si>
+    <t>VMB3096</t>
+  </si>
+  <si>
+    <t>050602-14-0461</t>
+  </si>
+  <si>
+    <t>JWC2377</t>
+  </si>
+  <si>
+    <t>051107-01-1093</t>
+  </si>
+  <si>
+    <t>JTD5106</t>
+  </si>
+  <si>
+    <t>660507-04-5309</t>
+  </si>
+  <si>
+    <t>TCN6958</t>
+  </si>
+  <si>
+    <t>020718-10-1635</t>
+  </si>
+  <si>
+    <t>MDF3352</t>
+  </si>
+  <si>
+    <t>820807-04-5001</t>
+  </si>
+  <si>
+    <t>BNL8065</t>
+  </si>
+  <si>
+    <t>800623-03-5708</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -195,8 +306,14 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -206,6 +323,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -278,16 +407,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
+      <right style="thin">
+        <color rgb="FF000000"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
+      <top style="thin">
+        <color rgb="FF000000"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -295,7 +424,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -309,9 +438,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -626,16 +758,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{689C8A9F-98AE-49F8-89B3-BABBB35DE82F}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.36328125" customWidth="1"/>
     <col min="2" max="2" width="17.36328125" customWidth="1"/>
     <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -643,13 +774,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
@@ -657,201 +785,347 @@
         <v>3</v>
       </c>
       <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
+      <c r="B4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="3" t="s">
+      <c r="C14" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
+      <c r="B18" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="C18" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
+      <c r="B19" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="C19" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
+      <c r="B20" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="C20" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="1"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="10"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A34" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" s="9"/>
+      <c r="B43" s="9"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A24:B24"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated Stability excel sheet
</commit_message>
<xml_diff>
--- a/pages/STPTestData.xlsx
+++ b/pages/STPTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B45F971-E757-4F9D-922F-8306264F86BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AEB3E82-CD7A-4AAF-AD1B-798925616DDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{45C1E7C0-1AF2-45CB-BEA8-DD612E61CE1D}"/>
   </bookViews>
@@ -889,10 +889,10 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="1" t="s">

</xml_diff>